<commit_message>
Add factory/field split to 의왕초평 기성청구현황
5회차 실제값 기준 공장(제1사업장) 58.97% / 현장(제2사업장) 41.03% 비율 산정,
1~4회차에 동일 비율 적용하여 공장분/현장분 금액 및 비율 컬럼 추가

https://claude.ai/code/session_015azLbSeBDQKuTi2QuFhHS4
</commit_message>
<xml_diff>
--- a/의왕초평_도급기성청구현황.xlsx
+++ b/의왕초평_도급기성청구현황.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,24 @@
     </font>
     <font>
       <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00843C0C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="9"/>
@@ -52,6 +70,36 @@
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00843C0C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
@@ -68,14 +116,9 @@
     </font>
     <font>
       <name val="맑은 고딕"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
@@ -96,7 +139,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +158,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
@@ -125,12 +183,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F9F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBF3FA"/>
+        <fgColor rgb="00843C0C"/>
       </patternFill>
     </fill>
   </fills>
@@ -152,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -160,89 +238,136 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -610,459 +735,585 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>의왕초평 A-4BL  도급 기성청구 현황</t>
+          <t>의왕초평 A-4BL  도급 기성청구 현황 (공장/현장 분리)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>계약금액 (도급기성청구 소계)</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>86000000000</v>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>※ 추가정산 포함 총계약 90,000,000,000원  /  단위 : 원, VAT포함</t>
+          <t>【공장/현장 분리 기준 비율】</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>공장(제1사업장): 2,347,000,000원</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>현장(제2사업장): 1,633,000,000원</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>기준합계: 3,980,000,000원</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>※ 5회차 실제 데이터 기준 비율 / 1~4회차는 동일 비율 적용 (추정)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>기본정보</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>기본정보</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>공장(제1사업장)
+58.97%</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>현장(제2사업장)
+41.03%</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>금회합계</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>업체별 금회금액</t>
+        </is>
+      </c>
+      <c r="Q3" s="7" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>회차</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>구분
-(정식/약식)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>정식
+/약식</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>품의번호</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>기안일자</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>처리일자
-(총괄표 기준)</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>처리일자</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>청구월</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>금회금액
-(합계)</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>공장분
+금액</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>공장
+비율</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>현장분
+금액</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>현장
+비율</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>합 계</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>극동건설(주)
 51%</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>(주)HJ중공업
 15%</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>(주)서한
 14%</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
         <is>
           <t>(주)대저건설
 10%</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="P4" s="9" t="inlineStr">
         <is>
           <t>(주)엔알비
 10%</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>누계금액</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>1회</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>정식</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>(주)엔알비-2025-17478</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>2025-11-29</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>2025년 12월</t>
         </is>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G5" s="18" t="n">
+        <v>2993309548</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>0.5896984925137904</v>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>2082690452</v>
+      </c>
+      <c r="J5" s="21" t="n">
+        <v>0.4103015074862096</v>
+      </c>
+      <c r="K5" s="22" t="n">
         <v>5076000000</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="L5" s="23" t="n">
         <v>2588760000</v>
       </c>
-      <c r="I4" s="11" t="n">
+      <c r="M5" s="23" t="n">
         <v>761400000</v>
       </c>
-      <c r="J4" s="11" t="n">
+      <c r="N5" s="23" t="n">
         <v>710640000</v>
       </c>
-      <c r="K4" s="11" t="n">
+      <c r="O5" s="23" t="n">
         <v>507600000</v>
       </c>
-      <c r="L4" s="11" t="n">
+      <c r="P5" s="23" t="n">
         <v>507600000</v>
       </c>
-      <c r="M4" s="12" t="n">
-        <v>5076000000</v>
-      </c>
-      <c r="N4" s="8" t="inlineStr">
+      <c r="Q5" s="24" t="inlineStr">
         <is>
           <t>기안일(11/29) vs 처리일(12/04) 월 상이</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>2회</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>약식</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>(주)엔알비-2026-1859</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D6" s="28" t="inlineStr">
         <is>
           <t>2026-02-02</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>2026-02-04</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F6" s="29" t="inlineStr">
         <is>
           <t>2026년 2월</t>
         </is>
       </c>
-      <c r="G5" s="17" t="n">
+      <c r="G6" s="18" t="n">
+        <v>367971859</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>0.5896984919871795</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>256028141</v>
+      </c>
+      <c r="J6" s="21" t="n">
+        <v>0.4103015080128205</v>
+      </c>
+      <c r="K6" s="22" t="n">
         <v>624000000</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="L6" s="30" t="n">
         <v>318240000</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="M6" s="30" t="n">
         <v>93600000</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="N6" s="30" t="n">
         <v>87360000</v>
       </c>
-      <c r="K5" s="18" t="n">
+      <c r="O6" s="30" t="n">
         <v>62400000</v>
       </c>
-      <c r="L5" s="18" t="n">
+      <c r="P6" s="30" t="n">
         <v>62400000</v>
       </c>
-      <c r="M5" s="19" t="n">
-        <v>5700000000</v>
-      </c>
-      <c r="N5" s="15" t="inlineStr"/>
+      <c r="Q6" s="31" t="inlineStr"/>
     </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>3회</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
           <t>약식</t>
         </is>
       </c>
-      <c r="C6" s="22" t="inlineStr">
+      <c r="C7" s="34" t="inlineStr">
         <is>
           <t>(주)엔알비-2026-4026</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
+      <c r="D7" s="35" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="E6" s="22" t="inlineStr">
+      <c r="E7" s="35" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="F6" s="23" t="inlineStr">
+      <c r="F7" s="36" t="inlineStr">
         <is>
           <t>2026년 3월</t>
         </is>
       </c>
-      <c r="G6" s="24" t="n">
+      <c r="G7" s="18" t="n">
+        <v>967105528</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>0.5896984926829268</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <v>672894472</v>
+      </c>
+      <c r="J7" s="21" t="n">
+        <v>0.4103015073170732</v>
+      </c>
+      <c r="K7" s="22" t="n">
         <v>1640000000</v>
       </c>
-      <c r="H6" s="25" t="n">
+      <c r="L7" s="37" t="n">
         <v>836400000</v>
       </c>
-      <c r="I6" s="25" t="n">
+      <c r="M7" s="37" t="n">
         <v>246000000</v>
       </c>
-      <c r="J6" s="25" t="n">
+      <c r="N7" s="37" t="n">
         <v>229600000</v>
       </c>
-      <c r="K6" s="25" t="n">
+      <c r="O7" s="37" t="n">
         <v>164000000</v>
       </c>
-      <c r="L6" s="25" t="n">
+      <c r="P7" s="37" t="n">
         <v>164000000</v>
       </c>
-      <c r="M6" s="26" t="n">
-        <v>7340000000</v>
-      </c>
-      <c r="N6" s="22" t="inlineStr"/>
+      <c r="Q7" s="38" t="inlineStr"/>
     </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>4회</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>정식</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>(주)엔알비-2026-5251</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>2026-04-06</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>2026년 4월</t>
         </is>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G8" s="18" t="n">
+        <v>1727816583</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>0.5896984924914676</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>1202183417</v>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>0.4103015075085324</v>
+      </c>
+      <c r="K8" s="22" t="n">
         <v>2930000000</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="L8" s="23" t="n">
         <v>1494300000</v>
       </c>
-      <c r="I7" s="11" t="n">
+      <c r="M8" s="23" t="n">
         <v>439500000</v>
       </c>
-      <c r="J7" s="11" t="n">
+      <c r="N8" s="23" t="n">
         <v>410200000</v>
       </c>
-      <c r="K7" s="11" t="n">
+      <c r="O8" s="23" t="n">
         <v>293000000</v>
       </c>
-      <c r="L7" s="11" t="n">
+      <c r="P8" s="23" t="n">
         <v>293000000</v>
       </c>
-      <c r="M7" s="12" t="n">
-        <v>10270000000</v>
-      </c>
-      <c r="N7" s="8" t="inlineStr">
+      <c r="Q8" s="24" t="inlineStr">
         <is>
           <t>기안일(3/25) vs 처리일(4/06) 월 상이</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>5회</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>약식</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>(주)엔알비-2026-7755</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>미확인</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>2026년 5월</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>3980000000</v>
-      </c>
-      <c r="H8" s="11" t="n">
-        <v>2029800000</v>
-      </c>
-      <c r="I8" s="11" t="n">
-        <v>597000000</v>
-      </c>
-      <c r="J8" s="11" t="n">
-        <v>557200000</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>398000000</v>
-      </c>
-      <c r="L8" s="11" t="n">
-        <v>398000000</v>
-      </c>
-      <c r="M8" s="12" t="n">
-        <v>14250000000</v>
-      </c>
-      <c r="N8" s="8" t="inlineStr">
-        <is>
-          <t>기안서 1p 누락 – 처리일은 총괄표 기준</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>5회</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>약식</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="inlineStr">
+        <is>
+          <t>(주)엔알비-2026-7755</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="F9" s="36" t="inlineStr">
+        <is>
+          <t>2026년 5월</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>2347000000</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>0.5896984924623115</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>1633000000</v>
+      </c>
+      <c r="J9" s="21" t="n">
+        <v>0.4103015075376885</v>
+      </c>
+      <c r="K9" s="22" t="n">
+        <v>3980000000</v>
+      </c>
+      <c r="L9" s="37" t="n">
+        <v>2029800000</v>
+      </c>
+      <c r="M9" s="37" t="n">
+        <v>597000000</v>
+      </c>
+      <c r="N9" s="37" t="n">
+        <v>557200000</v>
+      </c>
+      <c r="O9" s="37" t="n">
+        <v>398000000</v>
+      </c>
+      <c r="P9" s="37" t="n">
+        <v>398000000</v>
+      </c>
+      <c r="Q9" s="38" t="inlineStr">
+        <is>
+          <t>5회차 실제값 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>합   계</t>
         </is>
       </c>
-      <c r="G9" s="29">
-        <f>SUM(G4:G8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="29">
-        <f>SUM(H4:H8)</f>
-        <v/>
-      </c>
-      <c r="I9" s="29">
-        <f>SUM(I4:I8)</f>
-        <v/>
-      </c>
-      <c r="J9" s="29">
-        <f>SUM(J4:J8)</f>
-        <v/>
-      </c>
-      <c r="K9" s="29">
-        <f>SUM(K4:K8)</f>
-        <v/>
-      </c>
-      <c r="L9" s="29">
-        <f>SUM(L4:L8)</f>
-        <v/>
-      </c>
-      <c r="M9" s="29" t="n">
+      <c r="G10" s="40" t="n">
+        <v>8403203518</v>
+      </c>
+      <c r="H10" s="41" t="n">
+        <v>0.5896984924912281</v>
+      </c>
+      <c r="I10" s="42" t="n">
+        <v>5846796482</v>
+      </c>
+      <c r="J10" s="43" t="n">
+        <v>0.4103015075087719</v>
+      </c>
+      <c r="K10" s="44" t="n">
         <v>14250000000</v>
       </c>
-      <c r="N9" s="30" t="inlineStr"/>
+      <c r="L10" s="44" t="n">
+        <v>7267500000</v>
+      </c>
+      <c r="M10" s="44" t="n">
+        <v>2137500000</v>
+      </c>
+      <c r="N10" s="44" t="n">
+        <v>1995000000</v>
+      </c>
+      <c r="O10" s="44" t="n">
+        <v>1425000000</v>
+      </c>
+      <c r="P10" s="44" t="n">
+        <v>1425000000</v>
+      </c>
+      <c r="Q10" s="45" t="inlineStr"/>
     </row>
-    <row r="11">
-      <c r="A11" s="31" t="inlineStr">
-        <is>
-          <t>※ 청구월은 사업비회수금 총괄표의 처리일자 기준.  1회(기안 11/29→처리 12/04), 4회(기안 3/25→처리 4/06)는 기안월과 처리월이 상이함.</t>
+    <row r="12">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>※ 공장(제1사업장) 58.97% / 현장(제2사업장) 41.03%  ← 5회차 실제값(공장 2,347,000,000원 / 현장 1,633,000,000원 / 합계 3,980,000,000원) 기준 산정. 1~4회차는 동일 비율 추정 적용.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="H2:N2"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A11:N11"/>
-    <mergeCell ref="A1:N1"/>
+  <mergeCells count="13">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="L3:P3"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="A12:Q12"/>
+    <mergeCell ref="K2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="L2:Q2"/>
+    <mergeCell ref="I3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add 4회차 payment history section to 의왕초평 기성청구현황
4회차 업체별 입금 현황 추가:
- 4월: 대저건설(4/24) + 엔알비(4/23) = 586,000,000원
- 5월: 극동건설(5/7) + 서한(5/7) = 1,904,500,000원
- 미수금: HJ중공업 439,500,000원

https://claude.ai/code/session_015azLbSeBDQKuTi2QuFhHS4
</commit_message>
<xml_diff>
--- a/의왕초평_도급기성청구현황.xlsx
+++ b/의왕초평_도급기성청구현황.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="30">
     <font>
       <name val="맑은 고딕"/>
       <family val="2"/>
@@ -114,8 +114,108 @@
       <color theme="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00843C0C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <i val="1"/>
+      <color rgb="00375623"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00843C0C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -144,8 +244,53 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -212,6 +357,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
@@ -219,7 +370,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -267,6 +418,120 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="23" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="25" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="27" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="28" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="27" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="27" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -633,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="7" customWidth="1" style="5" min="1" max="1"/>
@@ -1185,9 +1450,325 @@
       </c>
       <c r="I18" s="4" t="n"/>
     </row>
+    <row r="21" ht="30" customHeight="1" s="5">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>【 4회차 입금 현황 】</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1" s="5">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>업체명</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>청구금액</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>4월 입금</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>4월
+입금일</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>5월 입금</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>5월
+입금일</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t>입금합계</t>
+        </is>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
+        <is>
+          <t>미수금</t>
+        </is>
+      </c>
+      <c r="I22" s="20" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" s="5">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>극동건설(주)</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="n">
+        <v>1494300000</v>
+      </c>
+      <c r="C23" s="27" t="n"/>
+      <c r="D23" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="n">
+        <v>1494300000</v>
+      </c>
+      <c r="F23" s="30" t="inlineStr">
+        <is>
+          <t>5/7</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="n">
+        <v>1494300000</v>
+      </c>
+      <c r="H23" s="32" t="n"/>
+      <c r="I23" s="33" t="inlineStr">
+        <is>
+          <t>완납</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" s="5">
+      <c r="A24" s="34" t="inlineStr">
+        <is>
+          <t>(주)HJ중공업</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n">
+        <v>439500000</v>
+      </c>
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="36" t="n"/>
+      <c r="F24" s="30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="37" t="n"/>
+      <c r="H24" s="38" t="n">
+        <v>439500000</v>
+      </c>
+      <c r="I24" s="39" t="inlineStr">
+        <is>
+          <t>미수금</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" s="5">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>(주)서한</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="n">
+        <v>410200000</v>
+      </c>
+      <c r="C25" s="27" t="n"/>
+      <c r="D25" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="n">
+        <v>410200000</v>
+      </c>
+      <c r="F25" s="30" t="inlineStr">
+        <is>
+          <t>5/7</t>
+        </is>
+      </c>
+      <c r="G25" s="31" t="n">
+        <v>410200000</v>
+      </c>
+      <c r="H25" s="32" t="n"/>
+      <c r="I25" s="33" t="inlineStr">
+        <is>
+          <t>완납</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" s="5">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>(주)대저건설</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="n">
+        <v>293000000</v>
+      </c>
+      <c r="C26" s="42" t="n">
+        <v>293000000</v>
+      </c>
+      <c r="D26" s="28" t="inlineStr">
+        <is>
+          <t>4/24</t>
+        </is>
+      </c>
+      <c r="E26" s="36" t="n"/>
+      <c r="F26" s="30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="31" t="n">
+        <v>293000000</v>
+      </c>
+      <c r="H26" s="32" t="n"/>
+      <c r="I26" s="43" t="inlineStr">
+        <is>
+          <t>완납</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1" s="5">
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>(주)엔알비(LH)</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="n">
+        <v>293000000</v>
+      </c>
+      <c r="C27" s="42" t="n">
+        <v>293000000</v>
+      </c>
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>4/23</t>
+        </is>
+      </c>
+      <c r="E27" s="36" t="n"/>
+      <c r="F27" s="30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="31" t="n">
+        <v>293000000</v>
+      </c>
+      <c r="H27" s="32" t="n"/>
+      <c r="I27" s="33" t="inlineStr">
+        <is>
+          <t>완납</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1" s="5">
+      <c r="A28" s="44" t="inlineStr">
+        <is>
+          <t>합   계</t>
+        </is>
+      </c>
+      <c r="B28" s="45" t="n">
+        <v>2930000000</v>
+      </c>
+      <c r="C28" s="46" t="n">
+        <v>586000000</v>
+      </c>
+      <c r="D28" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="48" t="n">
+        <v>1904500000</v>
+      </c>
+      <c r="F28" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="50" t="n">
+        <v>2490500000</v>
+      </c>
+      <c r="H28" s="51" t="n">
+        <v>439500000</v>
+      </c>
+      <c r="I28" s="44" t="inlineStr"/>
+    </row>
+    <row r="30" ht="22" customHeight="1" s="5">
+      <c r="A30" s="52" t="inlineStr">
+        <is>
+          <t>▶ 월별 입금 요약</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" s="5">
+      <c r="A31" s="47" t="inlineStr">
+        <is>
+          <t>4월</t>
+        </is>
+      </c>
+      <c r="B31" s="53" t="n">
+        <v>586000000</v>
+      </c>
+      <c r="D31" s="54" t="inlineStr">
+        <is>
+          <t>대저건설(4/24 293,000,000) + 엔알비(4/23 293,000,000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" s="5">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>5월</t>
+        </is>
+      </c>
+      <c r="B32" s="55" t="n">
+        <v>1904500000</v>
+      </c>
+      <c r="D32" s="54" t="inlineStr">
+        <is>
+          <t>극동건설(5/7 1,494,300,000) + 서한(5/7 410,200,000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" s="5">
+      <c r="A33" s="56" t="inlineStr">
+        <is>
+          <t>미수금</t>
+        </is>
+      </c>
+      <c r="B33" s="51" t="n">
+        <v>439500000</v>
+      </c>
+      <c r="D33" s="54" t="inlineStr">
+        <is>
+          <t>(주)HJ중공업 미입금</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="13">
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="A31"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="D31:I31"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="A28"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A33"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>

</xml_diff>